<commit_message>
feat: use wind json for ratingdog downloads
</commit_message>
<xml_diff>
--- a/skills/download-private-bond/assets/公式模板.xlsx
+++ b/skills/download-private-bond/assets/公式模板.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\LLMproject\DownloadPrivateBond\skills\download-private-bond\assets\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DA4CEEFA-A618-40EE-97B0-EEE878B23CA1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4D6AECC9-41F8-4FD8-A444-626031F658D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-25710" yWindow="-110" windowWidth="25820" windowHeight="13900" xr2:uid="{BACEADC3-2DF2-43AF-A933-7F7F1B3EB297}"/>
+    <workbookView xWindow="2280" yWindow="2280" windowWidth="25800" windowHeight="9920" xr2:uid="{BACEADC3-2DF2-43AF-A933-7F7F1B3EB297}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -451,20 +451,20 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E7B19218-A3E4-458D-8AF5-682A7F84AF8E}">
   <dimension ref="A1:E2"/>
-  <sheetFormatPr defaultRowHeight="14.15" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultRowHeight="14" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="37.140625" customWidth="1"/>
-    <col min="2" max="2" width="17.92578125" customWidth="1"/>
-    <col min="3" max="3" width="27.0703125" customWidth="1"/>
+    <col min="1" max="1" width="17.9140625" customWidth="1"/>
+    <col min="2" max="2" width="37.1640625" customWidth="1"/>
+    <col min="3" max="3" width="27.08203125" customWidth="1"/>
     <col min="4" max="4" width="84.5" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B1" t="s">
         <v>0</v>
-      </c>
-      <c r="B1" t="s">
-        <v>1</v>
       </c>
       <c r="C1" t="s">
         <v>2</v>
@@ -476,16 +476,16 @@
         <v>5</v>
       </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.35">
-      <c r="A2" t="str">
+    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A2" t="s">
+        <v>4</v>
+      </c>
+      <c r="B2" t="str">
         <f>[1]!s_info_compname(C2)</f>
         <v>乐山国有资产投资运营(集团)有限公司</v>
       </c>
-      <c r="B2" t="s">
-        <v>4</v>
-      </c>
       <c r="C2" t="str">
-        <f>[1]!to_windcode(B2)</f>
+        <f>[1]!to_windcode(A2)</f>
         <v>282882.SH</v>
       </c>
       <c r="D2" t="str">

</xml_diff>